<commit_message>
fix(gen): align the P_BUS router workbook with the contract
PBUS_APB_DEC.xlsx: input width 18 (meta.pbus_paddr_width), slave width 14
(meta.apb_paddr_width), offsets relative to apb_window_base. m_qnsc_p_bus_dec
regenerated. The wrapper no longer instantiates the router; the files stay for
whoever builds P_BUS.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/util/gen/p_bus_apb_dec/PBUS_APB_DEC.xlsx
+++ b/util/gen/p_bus_apb_dec/PBUS_APB_DEC.xlsx
@@ -502,11 +502,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>P_BUS's i_paddr width -- carries the full absolute 32-bit system address (axi_lite_to_apb passes AXI addr through unmodified; s_bus_pkg's own APB rule already matches on the absolute AXI2APB window base).</t>
+          <t>P_BUS's i_paddr width: the offset inside the 256 KiB AXI2APB window (util/qsoc_contract.yml meta.pbus_paddr_width). m_qnsc_wrap_bus passes the low 18 bits of the AXI address, so OFFSET and END ADDRESS below are relative to the window base (meta.apb_window_base).</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFFFFFFFF</t>
+          <t>0x3FFFF</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -653,11 +653,11 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0x80000000</t>
+          <t>0x00000</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0x80003FFF</t>
+          <t>0x03FFF</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -686,11 +686,11 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0x80004000</t>
+          <t>0x04000</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0x80007FFF</t>
+          <t>0x07FFF</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -719,11 +719,11 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0x80008000</t>
+          <t>0x08000</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0x8000BFFF</t>
+          <t>0x0BFFF</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -752,11 +752,11 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0x8000C000</t>
+          <t>0x0C000</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0x8000FFFF</t>
+          <t>0x0FFFF</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -785,11 +785,11 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0x80010000</t>
+          <t>0x10000</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0x80013FFF</t>
+          <t>0x13FFF</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -818,11 +818,11 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0x80014000</t>
+          <t>0x14000</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0x80017FFF</t>
+          <t>0x17FFF</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -851,11 +851,11 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0x80018000</t>
+          <t>0x18000</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0x8001BFFF</t>
+          <t>0x1BFFF</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -884,11 +884,11 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0x8001C000</t>
+          <t>0x1C000</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0x8001FFFF</t>
+          <t>0x1FFFF</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0x80020000</t>
+          <t>0x20000</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0x80023FFF</t>
+          <t>0x23FFF</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -950,11 +950,11 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0x80024000</t>
+          <t>0x24000</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0x80027FFF</t>
+          <t>0x27FFF</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -983,11 +983,11 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0x80028000</t>
+          <t>0x28000</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0x8002BFFF</t>
+          <t>0x2BFFF</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1016,11 +1016,11 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0x8002C000</t>
+          <t>0x2C000</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0x8002FFFF</t>
+          <t>0x2FFFF</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1049,11 +1049,11 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0x80030000</t>
+          <t>0x30000</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0x80033FFF</t>
+          <t>0x33FFF</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1082,11 +1082,11 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0x80034000</t>
+          <t>0x34000</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0x80037FFF</t>
+          <t>0x37FFF</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">

</xml_diff>